<commit_message>
add the dist excel and update the distance.py
</commit_message>
<xml_diff>
--- a/customer_table.xlsx
+++ b/customer_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="123820"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pawan\Desktop\og\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\og\og-excel-to-sql\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{348579EC-71D2-4473-B9B1-D9D9E59059D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{165590E4-29FF-4EDE-ACCE-68F5F155F021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1440" yWindow="1185" windowWidth="24570" windowHeight="13830" tabRatio="907" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-210" yWindow="0" windowWidth="14715" windowHeight="15600" tabRatio="907" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -6635,6 +6635,7 @@
         <sz val="6"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>Spectrum</t>
     </r>
@@ -6643,14 +6644,16 @@
         <sz val="6"/>
         <color rgb="FF000000"/>
         <rFont val="Times New Roman"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>Tool</t>
     </r>
@@ -6659,14 +6662,16 @@
         <sz val="6"/>
         <color rgb="FF000000"/>
         <rFont val="Times New Roman"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>Engineers</t>
     </r>
@@ -6675,14 +6680,16 @@
         <sz val="6"/>
         <color rgb="FF000000"/>
         <rFont val="Times New Roman"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>(P)</t>
     </r>
@@ -6691,14 +6698,16 @@
         <sz val="6"/>
         <color rgb="FF000000"/>
         <rFont val="Times New Roman"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>Ltd</t>
     </r>
@@ -12630,7 +12639,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -12674,36 +12683,42 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="12"/>
@@ -12716,17 +12731,20 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="12"/>
@@ -12753,16 +12771,6 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="6"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="6"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
     </font>
   </fonts>
   <fills count="13">
@@ -13868,24 +13876,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -13901,6 +13891,24 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -13910,27 +13918,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill>
@@ -13991,100 +13979,12 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -14387,7 +14287,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:AB102"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="3.42578125" style="1" customWidth="1"/>
     <col min="2" max="3" width="29.42578125" style="5" customWidth="1"/>
@@ -14417,7 +14317,7 @@
     <col min="28" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:28" s="16" customFormat="1" ht="15" customHeight="1">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -14503,7 +14403,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:28" ht="15" customHeight="1">
       <c r="A2" s="7">
         <v>1</v>
       </c>
@@ -14588,7 +14488,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:28" ht="15" customHeight="1">
       <c r="A3" s="7">
         <v>2</v>
       </c>
@@ -14671,7 +14571,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:28" ht="15" customHeight="1">
       <c r="A4" s="7">
         <v>3</v>
       </c>
@@ -14754,7 +14654,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:28" ht="15" customHeight="1">
       <c r="A5" s="7">
         <v>4</v>
       </c>
@@ -14839,7 +14739,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:28" ht="15" customHeight="1">
       <c r="A6" s="7">
         <v>5</v>
       </c>
@@ -14922,7 +14822,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:28" ht="15" customHeight="1">
       <c r="A7" s="7">
         <v>7</v>
       </c>
@@ -15005,7 +14905,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:28" ht="15" customHeight="1">
       <c r="A8" s="7">
         <v>8</v>
       </c>
@@ -15090,7 +14990,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:28" ht="15" customHeight="1">
       <c r="A9" s="7">
         <v>9</v>
       </c>
@@ -15177,7 +15077,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:28" ht="15" customHeight="1">
       <c r="A10" s="7">
         <v>6</v>
       </c>
@@ -15264,7 +15164,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:28" ht="15" customHeight="1">
       <c r="A11" s="7">
         <v>10</v>
       </c>
@@ -15349,7 +15249,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:28" ht="15" customHeight="1">
       <c r="A12" s="7">
         <v>11</v>
       </c>
@@ -15434,7 +15334,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="13" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:28" ht="15" customHeight="1">
       <c r="A13" s="7">
         <v>12</v>
       </c>
@@ -15519,7 +15419,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="14" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:28" ht="15" customHeight="1">
       <c r="A14" s="7">
         <v>13</v>
       </c>
@@ -15602,7 +15502,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="15" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:28" ht="15" customHeight="1">
       <c r="A15" s="7">
         <v>14</v>
       </c>
@@ -15685,7 +15585,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="16" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:28" ht="15" customHeight="1">
       <c r="A16" s="7">
         <v>15</v>
       </c>
@@ -15770,7 +15670,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:28" ht="15" customHeight="1">
       <c r="A17" s="7">
         <v>16</v>
       </c>
@@ -15855,7 +15755,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:28" ht="15" customHeight="1">
       <c r="A18" s="7">
         <v>17</v>
       </c>
@@ -15942,7 +15842,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:28" ht="15" customHeight="1">
       <c r="A19" s="7">
         <v>18</v>
       </c>
@@ -16027,7 +15927,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:28" ht="15" customHeight="1">
       <c r="A20" s="7">
         <v>19</v>
       </c>
@@ -16112,7 +16012,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:28" ht="15" customHeight="1">
       <c r="A21" s="7">
         <v>20</v>
       </c>
@@ -16197,7 +16097,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:28" ht="15" customHeight="1">
       <c r="A22" s="7">
         <v>21</v>
       </c>
@@ -16284,7 +16184,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:28" ht="15" customHeight="1">
       <c r="A23" s="7">
         <v>22</v>
       </c>
@@ -16367,7 +16267,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="24" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:28" ht="15" customHeight="1">
       <c r="A24" s="7">
         <v>23</v>
       </c>
@@ -16452,7 +16352,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:28" ht="15" customHeight="1">
       <c r="A25" s="7">
         <v>24</v>
       </c>
@@ -16537,7 +16437,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:28" ht="15" customHeight="1">
       <c r="A26" s="7">
         <v>25</v>
       </c>
@@ -16622,7 +16522,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="27" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:28" ht="15" customHeight="1">
       <c r="A27" s="7">
         <v>26</v>
       </c>
@@ -16703,7 +16603,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:28" ht="15" customHeight="1">
       <c r="A28" s="7">
         <v>27</v>
       </c>
@@ -16788,7 +16688,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="29" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:28" ht="15" customHeight="1">
       <c r="A29" s="7">
         <v>28</v>
       </c>
@@ -16873,7 +16773,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="30" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:28" ht="15" customHeight="1">
       <c r="A30" s="7">
         <v>29</v>
       </c>
@@ -16958,7 +16858,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="31" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:28" ht="15" customHeight="1">
       <c r="A31" s="7">
         <v>30</v>
       </c>
@@ -17041,7 +16941,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="32" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:28" ht="15" customHeight="1">
       <c r="A32" s="7">
         <v>31</v>
       </c>
@@ -17126,7 +17026,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="33" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:28" ht="15" customHeight="1">
       <c r="A33" s="7">
         <v>32</v>
       </c>
@@ -17211,7 +17111,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="34" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:28" ht="15" customHeight="1">
       <c r="A34" s="7">
         <v>33</v>
       </c>
@@ -17294,7 +17194,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="35" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:28" ht="15" customHeight="1">
       <c r="A35" s="7">
         <v>34</v>
       </c>
@@ -17381,7 +17281,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="36" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:28" ht="15" customHeight="1">
       <c r="A36" s="7">
         <v>35</v>
       </c>
@@ -17464,7 +17364,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="37" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:28" ht="15" customHeight="1">
       <c r="A37" s="7">
         <v>36</v>
       </c>
@@ -17547,7 +17447,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="38" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:28" ht="15" customHeight="1">
       <c r="A38" s="7">
         <v>37</v>
       </c>
@@ -17632,7 +17532,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="39" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:28" ht="15" customHeight="1">
       <c r="A39" s="7">
         <v>38</v>
       </c>
@@ -17717,7 +17617,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="40" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:28" ht="15" customHeight="1">
       <c r="A40" s="7">
         <v>39</v>
       </c>
@@ -17804,7 +17704,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="41" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:28" ht="15" customHeight="1">
       <c r="A41" s="7">
         <v>40</v>
       </c>
@@ -17889,7 +17789,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="42" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:28" ht="15" customHeight="1">
       <c r="A42" s="7">
         <v>41</v>
       </c>
@@ -17976,7 +17876,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="43" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:28" ht="15" customHeight="1">
       <c r="A43" s="7">
         <v>42</v>
       </c>
@@ -18059,7 +17959,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="44" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:28" ht="15" customHeight="1">
       <c r="A44" s="7">
         <v>43</v>
       </c>
@@ -18144,7 +18044,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="45" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:28" ht="15" customHeight="1">
       <c r="A45" s="7">
         <v>44</v>
       </c>
@@ -18227,7 +18127,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="46" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:28" ht="15" customHeight="1">
       <c r="A46" s="7">
         <v>45</v>
       </c>
@@ -18310,7 +18210,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="47" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:28" ht="15" customHeight="1">
       <c r="A47" s="7">
         <v>46</v>
       </c>
@@ -18393,7 +18293,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="48" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:28" ht="15" customHeight="1">
       <c r="A48" s="7">
         <v>47</v>
       </c>
@@ -18478,7 +18378,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="49" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:28" ht="15" customHeight="1">
       <c r="A49" s="7">
         <v>48</v>
       </c>
@@ -18561,7 +18461,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="50" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:28" ht="15" customHeight="1">
       <c r="A50" s="7">
         <v>49</v>
       </c>
@@ -18644,7 +18544,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="51" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:28" ht="15" customHeight="1">
       <c r="A51" s="7">
         <v>50</v>
       </c>
@@ -18729,7 +18629,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="52" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:28" ht="15" customHeight="1">
       <c r="A52" s="7">
         <v>51</v>
       </c>
@@ -18812,7 +18712,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="53" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:28" ht="15" customHeight="1">
       <c r="A53" s="7">
         <v>52</v>
       </c>
@@ -18895,7 +18795,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="54" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:28" ht="15" customHeight="1">
       <c r="A54" s="7">
         <v>53</v>
       </c>
@@ -18980,7 +18880,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="55" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:28" ht="15" customHeight="1">
       <c r="A55" s="7">
         <v>54</v>
       </c>
@@ -19065,7 +18965,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="56" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:28" ht="15" customHeight="1">
       <c r="A56" s="7">
         <v>55</v>
       </c>
@@ -19150,7 +19050,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="57" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="57" spans="1:28" ht="15" customHeight="1">
       <c r="A57" s="7">
         <v>56</v>
       </c>
@@ -19235,7 +19135,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="58" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="58" spans="1:28" ht="15" customHeight="1">
       <c r="A58" s="7">
         <v>57</v>
       </c>
@@ -19318,7 +19218,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="59" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="59" spans="1:28" ht="15" customHeight="1">
       <c r="A59" s="7">
         <v>58</v>
       </c>
@@ -19401,7 +19301,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="60" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:28" ht="15" customHeight="1">
       <c r="A60" s="7">
         <v>59</v>
       </c>
@@ -19486,7 +19386,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="61" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="61" spans="1:28" ht="15" customHeight="1">
       <c r="A61" s="7">
         <v>60</v>
       </c>
@@ -19571,7 +19471,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="62" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="62" spans="1:28" ht="15" customHeight="1">
       <c r="A62" s="7">
         <v>61</v>
       </c>
@@ -19654,7 +19554,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="63" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="63" spans="1:28" ht="15" customHeight="1">
       <c r="A63" s="7">
         <v>62</v>
       </c>
@@ -19737,7 +19637,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="64" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="64" spans="1:28" ht="15" customHeight="1">
       <c r="A64" s="7">
         <v>63</v>
       </c>
@@ -19822,7 +19722,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="65" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:28" ht="15" customHeight="1">
       <c r="A65" s="7">
         <v>64</v>
       </c>
@@ -19907,7 +19807,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="66" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="66" spans="1:28" ht="15" customHeight="1">
       <c r="A66" s="7">
         <v>65</v>
       </c>
@@ -19994,7 +19894,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="67" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:28" ht="15" customHeight="1">
       <c r="A67" s="7">
         <v>66</v>
       </c>
@@ -20079,7 +19979,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="68" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="68" spans="1:28" ht="15" customHeight="1">
       <c r="A68" s="7">
         <v>67</v>
       </c>
@@ -20164,7 +20064,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="69" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="69" spans="1:28" ht="15" customHeight="1">
       <c r="A69" s="7">
         <v>68</v>
       </c>
@@ -20247,7 +20147,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="70" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="70" spans="1:28" ht="15" customHeight="1">
       <c r="A70" s="7">
         <v>69</v>
       </c>
@@ -20332,7 +20232,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="71" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="71" spans="1:28" ht="15" customHeight="1">
       <c r="A71" s="7">
         <v>70</v>
       </c>
@@ -20415,7 +20315,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="72" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="72" spans="1:28" ht="15" customHeight="1">
       <c r="A72" s="7">
         <v>71</v>
       </c>
@@ -20498,7 +20398,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="73" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="73" spans="1:28" ht="15" customHeight="1">
       <c r="A73" s="7">
         <v>72</v>
       </c>
@@ -20583,7 +20483,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="74" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="74" spans="1:28" ht="15" customHeight="1">
       <c r="A74" s="7">
         <v>73</v>
       </c>
@@ -20668,7 +20568,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="75" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="75" spans="1:28" ht="15" customHeight="1">
       <c r="A75" s="7">
         <v>74</v>
       </c>
@@ -20751,7 +20651,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="76" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="76" spans="1:28" ht="15" customHeight="1">
       <c r="A76" s="7">
         <v>75</v>
       </c>
@@ -20836,7 +20736,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="77" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="77" spans="1:28" ht="15" customHeight="1">
       <c r="A77" s="7">
         <v>76</v>
       </c>
@@ -20921,7 +20821,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="78" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="78" spans="1:28" ht="15" customHeight="1">
       <c r="A78" s="7">
         <v>77</v>
       </c>
@@ -21006,7 +20906,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="79" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="79" spans="1:28" ht="15" customHeight="1">
       <c r="A79" s="7">
         <v>78</v>
       </c>
@@ -21089,7 +20989,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="80" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="80" spans="1:28" ht="15" customHeight="1">
       <c r="A80" s="7">
         <v>79</v>
       </c>
@@ -21174,7 +21074,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="81" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="81" spans="1:28" ht="15" customHeight="1">
       <c r="A81" s="7">
         <v>80</v>
       </c>
@@ -21259,7 +21159,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="82" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="82" spans="1:28" ht="15" customHeight="1">
       <c r="A82" s="7">
         <v>81</v>
       </c>
@@ -21346,7 +21246,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="83" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="83" spans="1:28" ht="15" customHeight="1">
       <c r="A83" s="7">
         <v>82</v>
       </c>
@@ -21433,7 +21333,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="84" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="84" spans="1:28" ht="15" customHeight="1">
       <c r="A84" s="7">
         <v>83</v>
       </c>
@@ -21518,7 +21418,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="85" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="85" spans="1:28" ht="15" customHeight="1">
       <c r="A85" s="7">
         <v>84</v>
       </c>
@@ -21605,7 +21505,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="86" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="86" spans="1:28" ht="15" customHeight="1">
       <c r="A86" s="7">
         <v>85</v>
       </c>
@@ -21690,7 +21590,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="87" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="87" spans="1:28" ht="15" customHeight="1">
       <c r="A87" s="7">
         <v>86</v>
       </c>
@@ -21777,7 +21677,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="88" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="88" spans="1:28" ht="15" customHeight="1">
       <c r="A88" s="7">
         <v>87</v>
       </c>
@@ -21862,7 +21762,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="89" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="89" spans="1:28" ht="15" customHeight="1">
       <c r="A89" s="7">
         <v>88</v>
       </c>
@@ -21947,7 +21847,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="90" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="90" spans="1:28" ht="15" customHeight="1">
       <c r="A90" s="7">
         <v>89</v>
       </c>
@@ -22032,7 +21932,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="91" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="91" spans="1:28" ht="15" customHeight="1">
       <c r="A91" s="7">
         <v>90</v>
       </c>
@@ -22115,7 +22015,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="92" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="92" spans="1:28" ht="15" customHeight="1">
       <c r="A92" s="7">
         <v>91</v>
       </c>
@@ -22200,7 +22100,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="93" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="93" spans="1:28" ht="15" customHeight="1">
       <c r="A93" s="7">
         <v>92</v>
       </c>
@@ -22283,7 +22183,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="94" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="94" spans="1:28" ht="15" customHeight="1">
       <c r="A94" s="7">
         <v>93</v>
       </c>
@@ -22368,7 +22268,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="95" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="95" spans="1:28" ht="15" customHeight="1">
       <c r="A95" s="7">
         <v>94</v>
       </c>
@@ -22453,7 +22353,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="96" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="96" spans="1:28" ht="15" customHeight="1">
       <c r="A96" s="7">
         <v>95</v>
       </c>
@@ -22538,7 +22438,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="97" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="97" spans="1:28" ht="15" customHeight="1">
       <c r="A97" s="7">
         <v>96</v>
       </c>
@@ -22621,7 +22521,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="98" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="98" spans="1:28" ht="15" customHeight="1">
       <c r="A98" s="7">
         <v>97</v>
       </c>
@@ -22706,7 +22606,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="99" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="99" spans="1:28" ht="15" customHeight="1">
       <c r="A99" s="7">
         <v>98</v>
       </c>
@@ -22793,7 +22693,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="100" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="100" spans="1:28" ht="15" customHeight="1">
       <c r="A100" s="7">
         <v>99</v>
       </c>
@@ -22876,7 +22776,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="101" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="101" spans="1:28" ht="15" customHeight="1">
       <c r="A101" s="7">
         <v>100</v>
       </c>
@@ -22959,45 +22859,45 @@
         <v>637</v>
       </c>
     </row>
-    <row r="102" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="102" spans="1:28" ht="15" customHeight="1">
       <c r="A102" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="P27:Q27"/>
   </mergeCells>
+  <conditionalFormatting sqref="B1:C101">
+    <cfRule type="duplicateValues" dxfId="8" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D1:D101">
+    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="G1:G1048576">
-    <cfRule type="cellIs" dxfId="16" priority="36" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="36" operator="equal">
       <formula>"Calibration"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:J1048576">
-    <cfRule type="cellIs" dxfId="15" priority="127" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="127" operator="equal">
       <formula>"Warranty"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="128" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="128" operator="equal">
       <formula>"ACSC or Warranty"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="129" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="129" operator="equal">
       <formula>"Expired"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K10">
-    <cfRule type="cellIs" dxfId="12" priority="1423" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1423" operator="equal">
       <formula>"Warranty"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="1424" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="1424" operator="equal">
       <formula>"ACSC or Warranty"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="1425" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="1425" operator="equal">
       <formula>"Expired"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1:C101">
-    <cfRule type="duplicateValues" dxfId="9" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D1:D101">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.31496062992125984" right="0.31496062992125984" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="59" orientation="landscape" r:id="rId1"/>
@@ -23023,7 +22923,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5542F88-F753-4E30-BA51-29CEAE88F32C}">
   <dimension ref="A1:BA37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="2.140625" bestFit="1" customWidth="1"/>
@@ -23058,39 +22958,39 @@
     <col min="52" max="52" width="2.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:53" ht="15.75">
       <c r="A1" s="25"/>
       <c r="B1" s="26"/>
-      <c r="C1" s="181" t="s">
+      <c r="C1" s="188" t="s">
         <v>625</v>
       </c>
-      <c r="D1" s="181"/>
-      <c r="E1" s="182"/>
+      <c r="D1" s="188"/>
+      <c r="E1" s="189"/>
       <c r="F1" s="27"/>
       <c r="G1" s="28"/>
-      <c r="H1" s="181" t="s">
+      <c r="H1" s="188" t="s">
         <v>626</v>
       </c>
-      <c r="I1" s="181"/>
-      <c r="J1" s="181"/>
-      <c r="K1" s="182"/>
+      <c r="I1" s="188"/>
+      <c r="J1" s="188"/>
+      <c r="K1" s="189"/>
       <c r="L1" s="27"/>
       <c r="M1" s="28"/>
       <c r="N1" s="170"/>
-      <c r="O1" s="183" t="s">
+      <c r="O1" s="186" t="s">
         <v>627</v>
       </c>
-      <c r="P1" s="183"/>
-      <c r="Q1" s="183"/>
+      <c r="P1" s="186"/>
+      <c r="Q1" s="186"/>
       <c r="R1" s="29"/>
       <c r="S1" s="27"/>
       <c r="T1" s="28"/>
       <c r="U1" s="170"/>
-      <c r="V1" s="183" t="s">
+      <c r="V1" s="186" t="s">
         <v>628</v>
       </c>
-      <c r="W1" s="183"/>
-      <c r="X1" s="184"/>
+      <c r="W1" s="186"/>
+      <c r="X1" s="187"/>
       <c r="Y1" s="27"/>
       <c r="Z1" s="30"/>
       <c r="AA1" s="173"/>
@@ -23102,34 +23002,34 @@
       <c r="AE1" s="27"/>
       <c r="AF1" s="33"/>
       <c r="AG1" s="171"/>
-      <c r="AH1" s="185" t="s">
+      <c r="AH1" s="190" t="s">
         <v>630</v>
       </c>
-      <c r="AI1" s="185"/>
-      <c r="AJ1" s="186"/>
+      <c r="AI1" s="190"/>
+      <c r="AJ1" s="191"/>
       <c r="AK1" s="27"/>
       <c r="AL1" s="28"/>
       <c r="AM1" s="170"/>
-      <c r="AN1" s="183" t="s">
+      <c r="AN1" s="186" t="s">
         <v>631</v>
       </c>
-      <c r="AO1" s="183"/>
-      <c r="AP1" s="184"/>
+      <c r="AO1" s="186"/>
+      <c r="AP1" s="187"/>
       <c r="AQ1" s="27"/>
       <c r="AR1" s="30"/>
       <c r="AS1" s="173"/>
-      <c r="AT1" s="188" t="s">
+      <c r="AT1" s="182" t="s">
         <v>632</v>
       </c>
-      <c r="AU1" s="188"/>
-      <c r="AV1" s="189"/>
+      <c r="AU1" s="182"/>
+      <c r="AV1" s="183"/>
       <c r="AW1" s="34"/>
       <c r="AX1" s="34"/>
       <c r="AY1" s="34"/>
       <c r="AZ1" s="34"/>
       <c r="BA1" s="35"/>
     </row>
-    <row r="2" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:53" ht="15.75">
       <c r="A2" s="36" t="s">
         <v>12</v>
       </c>
@@ -23270,7 +23170,7 @@
       <c r="AZ2" s="55"/>
       <c r="BA2" s="35"/>
     </row>
-    <row r="3" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:53" ht="15.75">
       <c r="A3" s="62">
         <v>8</v>
       </c>
@@ -23411,7 +23311,7 @@
       <c r="AZ3" s="86"/>
       <c r="BA3" s="35"/>
     </row>
-    <row r="4" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:53" ht="15.75">
       <c r="A4" s="62">
         <v>8</v>
       </c>
@@ -23554,7 +23454,7 @@
       </c>
       <c r="BA4" s="35"/>
     </row>
-    <row r="5" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:53" ht="15.75">
       <c r="A5" s="62">
         <v>8</v>
       </c>
@@ -23697,7 +23597,7 @@
       </c>
       <c r="BA5" s="35"/>
     </row>
-    <row r="6" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:53" ht="15.75">
       <c r="A6" s="62">
         <v>8</v>
       </c>
@@ -23830,7 +23730,7 @@
       </c>
       <c r="BA6" s="35"/>
     </row>
-    <row r="7" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:53" ht="15.75">
       <c r="A7" s="62">
         <v>8</v>
       </c>
@@ -23953,7 +23853,7 @@
       </c>
       <c r="BA7" s="35"/>
     </row>
-    <row r="8" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:53" ht="15.75">
       <c r="A8" s="62">
         <v>8</v>
       </c>
@@ -24074,7 +23974,7 @@
       <c r="AZ8" s="86"/>
       <c r="BA8" s="35"/>
     </row>
-    <row r="9" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:53" ht="15.75">
       <c r="A9" s="62">
         <v>8</v>
       </c>
@@ -24195,7 +24095,7 @@
       <c r="AZ9" s="86"/>
       <c r="BA9" s="35"/>
     </row>
-    <row r="10" spans="1:53" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:53" ht="15" customHeight="1">
       <c r="A10" s="62">
         <v>8</v>
       </c>
@@ -24312,7 +24212,7 @@
       <c r="AZ10" s="34"/>
       <c r="BA10" s="35"/>
     </row>
-    <row r="11" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:53" ht="15.75">
       <c r="A11" s="62">
         <v>8</v>
       </c>
@@ -24429,7 +24329,7 @@
       <c r="AZ11" s="35"/>
       <c r="BA11" s="35"/>
     </row>
-    <row r="12" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:53" ht="15.75">
       <c r="A12" s="62">
         <v>8</v>
       </c>
@@ -24546,7 +24446,7 @@
       <c r="AZ12" s="35"/>
       <c r="BA12" s="35"/>
     </row>
-    <row r="13" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:53" ht="15.75">
       <c r="A13" s="62">
         <v>8</v>
       </c>
@@ -24663,7 +24563,7 @@
       <c r="AZ13" s="35"/>
       <c r="BA13" s="35"/>
     </row>
-    <row r="14" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:53" ht="15.75">
       <c r="A14" s="62">
         <v>8</v>
       </c>
@@ -24780,7 +24680,7 @@
       <c r="AZ14" s="35"/>
       <c r="BA14" s="35"/>
     </row>
-    <row r="15" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:53" ht="15.75">
       <c r="A15" s="62">
         <v>8</v>
       </c>
@@ -24875,7 +24775,7 @@
       <c r="AZ15" s="35"/>
       <c r="BA15" s="35"/>
     </row>
-    <row r="16" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:53" ht="15.75">
       <c r="A16" s="62">
         <v>8</v>
       </c>
@@ -24970,7 +24870,7 @@
       <c r="AZ16" s="35"/>
       <c r="BA16" s="35"/>
     </row>
-    <row r="17" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:53" ht="15.75">
       <c r="A17" s="62">
         <v>8</v>
       </c>
@@ -25067,7 +24967,7 @@
       <c r="AZ17" s="35"/>
       <c r="BA17" s="35"/>
     </row>
-    <row r="18" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:53" ht="15.75">
       <c r="A18" s="62">
         <v>8</v>
       </c>
@@ -25164,7 +25064,7 @@
       <c r="AZ18" s="35"/>
       <c r="BA18" s="35"/>
     </row>
-    <row r="19" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:53" ht="15.75">
       <c r="A19" s="62">
         <v>8</v>
       </c>
@@ -25261,7 +25161,7 @@
       <c r="AZ19" s="35"/>
       <c r="BA19" s="35"/>
     </row>
-    <row r="20" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:53" ht="15.75">
       <c r="A20" s="62">
         <v>8</v>
       </c>
@@ -25348,7 +25248,7 @@
       <c r="AZ20" s="35"/>
       <c r="BA20" s="35"/>
     </row>
-    <row r="21" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:53" ht="15.75">
       <c r="A21" s="62">
         <v>8</v>
       </c>
@@ -25418,8 +25318,8 @@
       <c r="AK21" s="100"/>
       <c r="AL21" s="100"/>
       <c r="AM21" s="100"/>
-      <c r="AN21" s="190"/>
-      <c r="AO21" s="190"/>
+      <c r="AN21" s="184"/>
+      <c r="AO21" s="184"/>
       <c r="AP21" s="100"/>
       <c r="AQ21" s="100"/>
       <c r="AR21" s="100"/>
@@ -25433,7 +25333,7 @@
       <c r="AZ21" s="35"/>
       <c r="BA21" s="35"/>
     </row>
-    <row r="22" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:53" ht="15.75">
       <c r="A22" s="62">
         <v>8</v>
       </c>
@@ -25518,7 +25418,7 @@
       <c r="AZ22" s="35"/>
       <c r="BA22" s="35"/>
     </row>
-    <row r="23" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:53" ht="15.75">
       <c r="A23" s="62">
         <v>8</v>
       </c>
@@ -25588,8 +25488,8 @@
       <c r="AK23" s="100"/>
       <c r="AL23" s="100"/>
       <c r="AM23" s="100"/>
-      <c r="AN23" s="190"/>
-      <c r="AO23" s="190"/>
+      <c r="AN23" s="184"/>
+      <c r="AO23" s="184"/>
       <c r="AP23" s="100"/>
       <c r="AQ23" s="100"/>
       <c r="AR23" s="100"/>
@@ -25603,7 +25503,7 @@
       <c r="AZ23" s="35"/>
       <c r="BA23" s="35"/>
     </row>
-    <row r="24" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:53" ht="15.75">
       <c r="A24" s="62">
         <v>8</v>
       </c>
@@ -25673,8 +25573,8 @@
       <c r="AK24" s="100"/>
       <c r="AL24" s="100"/>
       <c r="AM24" s="100"/>
-      <c r="AN24" s="190"/>
-      <c r="AO24" s="190"/>
+      <c r="AN24" s="184"/>
+      <c r="AO24" s="184"/>
       <c r="AP24" s="100"/>
       <c r="AQ24" s="100"/>
       <c r="AR24" s="100"/>
@@ -25688,7 +25588,7 @@
       <c r="AZ24" s="35"/>
       <c r="BA24" s="35"/>
     </row>
-    <row r="25" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:53" ht="15.75">
       <c r="A25" s="62">
         <v>8</v>
       </c>
@@ -25748,8 +25648,8 @@
       <c r="AK25" s="100"/>
       <c r="AL25" s="100"/>
       <c r="AM25" s="100"/>
-      <c r="AN25" s="190"/>
-      <c r="AO25" s="190"/>
+      <c r="AN25" s="184"/>
+      <c r="AO25" s="184"/>
       <c r="AP25" s="100"/>
       <c r="AQ25" s="100"/>
       <c r="AR25" s="100"/>
@@ -25763,7 +25663,7 @@
       <c r="AZ25" s="35"/>
       <c r="BA25" s="35"/>
     </row>
-    <row r="26" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:53" ht="15.75">
       <c r="A26" s="62">
         <v>8</v>
       </c>
@@ -25823,8 +25723,8 @@
       <c r="AK26" s="100"/>
       <c r="AL26" s="100"/>
       <c r="AM26" s="100"/>
-      <c r="AN26" s="191"/>
-      <c r="AO26" s="191"/>
+      <c r="AN26" s="185"/>
+      <c r="AO26" s="185"/>
       <c r="AP26" s="123"/>
       <c r="AQ26" s="123"/>
       <c r="AR26" s="123"/>
@@ -25838,7 +25738,7 @@
       <c r="AZ26" s="35"/>
       <c r="BA26" s="35"/>
     </row>
-    <row r="27" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:53" ht="15.75">
       <c r="A27" s="62">
         <v>8</v>
       </c>
@@ -25900,8 +25800,8 @@
       <c r="AK27" s="100"/>
       <c r="AL27" s="100"/>
       <c r="AM27" s="100"/>
-      <c r="AN27" s="191"/>
-      <c r="AO27" s="191"/>
+      <c r="AN27" s="185"/>
+      <c r="AO27" s="185"/>
       <c r="AP27" s="123"/>
       <c r="AQ27" s="123"/>
       <c r="AR27" s="123"/>
@@ -25915,7 +25815,7 @@
       <c r="AZ27" s="35"/>
       <c r="BA27" s="35"/>
     </row>
-    <row r="28" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:53" ht="15.75">
       <c r="A28" s="62">
         <v>8</v>
       </c>
@@ -25935,10 +25835,10 @@
       <c r="G28" s="100"/>
       <c r="H28" s="124"/>
       <c r="I28" s="124"/>
-      <c r="J28" s="191" t="s">
+      <c r="J28" s="185" t="s">
         <v>670</v>
       </c>
-      <c r="K28" s="191"/>
+      <c r="K28" s="185"/>
       <c r="L28" s="175"/>
       <c r="M28" s="175"/>
       <c r="N28" s="175"/>
@@ -25977,8 +25877,8 @@
       <c r="AK28" s="100"/>
       <c r="AL28" s="100"/>
       <c r="AM28" s="100"/>
-      <c r="AN28" s="191"/>
-      <c r="AO28" s="191"/>
+      <c r="AN28" s="185"/>
+      <c r="AO28" s="185"/>
       <c r="AP28" s="123"/>
       <c r="AQ28" s="123"/>
       <c r="AR28" s="123"/>
@@ -25992,7 +25892,7 @@
       <c r="AZ28" s="35"/>
       <c r="BA28" s="35"/>
     </row>
-    <row r="29" spans="1:53" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:53" ht="15.75">
       <c r="A29" s="128">
         <v>8</v>
       </c>
@@ -26057,7 +25957,7 @@
       <c r="AZ29" s="35"/>
       <c r="BA29" s="35"/>
     </row>
-    <row r="30" spans="1:53" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:53">
       <c r="A30" s="133"/>
       <c r="B30" s="133"/>
       <c r="C30" s="134"/>
@@ -26067,8 +25967,8 @@
       <c r="G30" s="136"/>
       <c r="H30" s="137"/>
       <c r="I30" s="137"/>
-      <c r="J30" s="187"/>
-      <c r="K30" s="187"/>
+      <c r="J30" s="181"/>
+      <c r="K30" s="181"/>
       <c r="L30" s="172"/>
       <c r="M30" s="172"/>
       <c r="N30" s="172"/>
@@ -26097,8 +25997,8 @@
       <c r="AK30" s="123"/>
       <c r="AL30" s="123"/>
       <c r="AM30" s="123"/>
-      <c r="AN30" s="191"/>
-      <c r="AO30" s="191"/>
+      <c r="AN30" s="185"/>
+      <c r="AO30" s="185"/>
       <c r="AP30" s="123"/>
       <c r="AQ30" s="123"/>
       <c r="AR30" s="123"/>
@@ -26112,7 +26012,7 @@
       <c r="AZ30" s="35"/>
       <c r="BA30" s="35"/>
     </row>
-    <row r="31" spans="1:53" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:53">
       <c r="A31" s="139"/>
       <c r="B31" s="139"/>
       <c r="C31" s="137"/>
@@ -26124,8 +26024,8 @@
         <v>671</v>
       </c>
       <c r="I31" s="137"/>
-      <c r="J31" s="187"/>
-      <c r="K31" s="187"/>
+      <c r="J31" s="181"/>
+      <c r="K31" s="181"/>
       <c r="L31" s="172"/>
       <c r="M31" s="172"/>
       <c r="N31" s="172"/>
@@ -26154,8 +26054,8 @@
       <c r="AK31" s="138"/>
       <c r="AL31" s="138"/>
       <c r="AM31" s="138"/>
-      <c r="AN31" s="187"/>
-      <c r="AO31" s="187"/>
+      <c r="AN31" s="181"/>
+      <c r="AO31" s="181"/>
       <c r="AP31" s="138"/>
       <c r="AQ31" s="138"/>
       <c r="AR31" s="138"/>
@@ -26169,7 +26069,7 @@
       <c r="AZ31" s="139"/>
       <c r="BA31" s="139"/>
     </row>
-    <row r="32" spans="1:53" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:53">
       <c r="A32" s="139"/>
       <c r="B32" s="139"/>
       <c r="C32" s="137"/>
@@ -26179,8 +26079,8 @@
       <c r="G32" s="138"/>
       <c r="H32" s="137"/>
       <c r="I32" s="137"/>
-      <c r="J32" s="187"/>
-      <c r="K32" s="187"/>
+      <c r="J32" s="181"/>
+      <c r="K32" s="181"/>
       <c r="L32" s="172"/>
       <c r="M32" s="172"/>
       <c r="N32" s="172"/>
@@ -26209,8 +26109,8 @@
       <c r="AK32" s="138"/>
       <c r="AL32" s="138"/>
       <c r="AM32" s="138"/>
-      <c r="AN32" s="187"/>
-      <c r="AO32" s="187"/>
+      <c r="AN32" s="181"/>
+      <c r="AO32" s="181"/>
       <c r="AP32" s="138"/>
       <c r="AQ32" s="138"/>
       <c r="AR32" s="138"/>
@@ -26224,7 +26124,7 @@
       <c r="AZ32" s="139"/>
       <c r="BA32" s="139"/>
     </row>
-    <row r="33" spans="1:53" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:53">
       <c r="A33" s="139"/>
       <c r="B33" s="139"/>
       <c r="C33" s="137"/>
@@ -26264,8 +26164,8 @@
       <c r="AK33" s="138"/>
       <c r="AL33" s="138"/>
       <c r="AM33" s="138"/>
-      <c r="AN33" s="187"/>
-      <c r="AO33" s="187"/>
+      <c r="AN33" s="181"/>
+      <c r="AO33" s="181"/>
       <c r="AP33" s="138"/>
       <c r="AQ33" s="138"/>
       <c r="AR33" s="138"/>
@@ -26279,7 +26179,7 @@
       <c r="AZ33" s="139"/>
       <c r="BA33" s="139"/>
     </row>
-    <row r="34" spans="1:53" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:53">
       <c r="A34" s="139"/>
       <c r="B34" s="139"/>
       <c r="C34" s="137"/>
@@ -26289,8 +26189,8 @@
       <c r="G34" s="138"/>
       <c r="H34" s="137"/>
       <c r="I34" s="137"/>
-      <c r="J34" s="187"/>
-      <c r="K34" s="187"/>
+      <c r="J34" s="181"/>
+      <c r="K34" s="181"/>
       <c r="L34" s="172"/>
       <c r="M34" s="172"/>
       <c r="N34" s="172"/>
@@ -26319,8 +26219,8 @@
       <c r="AK34" s="138"/>
       <c r="AL34" s="138"/>
       <c r="AM34" s="138"/>
-      <c r="AN34" s="187"/>
-      <c r="AO34" s="187"/>
+      <c r="AN34" s="181"/>
+      <c r="AO34" s="181"/>
       <c r="AP34" s="138"/>
       <c r="AQ34" s="138"/>
       <c r="AR34" s="138"/>
@@ -26334,13 +26234,13 @@
       <c r="AZ34" s="139"/>
       <c r="BA34" s="139"/>
     </row>
-    <row r="35" spans="1:53" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:53">
       <c r="F35" s="138"/>
       <c r="G35" s="138"/>
       <c r="H35" s="137"/>
       <c r="I35" s="137"/>
-      <c r="J35" s="187"/>
-      <c r="K35" s="187"/>
+      <c r="J35" s="181"/>
+      <c r="K35" s="181"/>
       <c r="L35" s="172"/>
       <c r="M35" s="172"/>
       <c r="N35" s="172"/>
@@ -26369,8 +26269,8 @@
       <c r="AK35" s="138"/>
       <c r="AL35" s="138"/>
       <c r="AM35" s="138"/>
-      <c r="AN35" s="187"/>
-      <c r="AO35" s="187"/>
+      <c r="AN35" s="181"/>
+      <c r="AO35" s="181"/>
       <c r="AP35" s="138"/>
       <c r="AQ35" s="138"/>
       <c r="AR35" s="138"/>
@@ -26384,7 +26284,7 @@
       <c r="AZ35" s="139"/>
       <c r="BA35" s="139"/>
     </row>
-    <row r="36" spans="1:53" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:53">
       <c r="F36" s="138"/>
       <c r="G36" s="138"/>
       <c r="H36" s="137"/>
@@ -26419,8 +26319,8 @@
       <c r="AK36" s="138"/>
       <c r="AL36" s="138"/>
       <c r="AM36" s="138"/>
-      <c r="AN36" s="187"/>
-      <c r="AO36" s="187"/>
+      <c r="AN36" s="181"/>
+      <c r="AO36" s="181"/>
       <c r="AP36" s="138"/>
       <c r="AQ36" s="138"/>
       <c r="AR36" s="138"/>
@@ -26434,7 +26334,7 @@
       <c r="AZ36" s="139"/>
       <c r="BA36" s="139"/>
     </row>
-    <row r="37" spans="1:53" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:53">
       <c r="F37" s="138"/>
       <c r="G37" s="138"/>
       <c r="H37" s="137"/>
@@ -26486,14 +26386,11 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="AN36:AO36"/>
-    <mergeCell ref="J32:K32"/>
-    <mergeCell ref="AN32:AO32"/>
-    <mergeCell ref="AN33:AO33"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="AN34:AO34"/>
-    <mergeCell ref="J35:K35"/>
-    <mergeCell ref="AN35:AO35"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="H1:K1"/>
+    <mergeCell ref="O1:Q1"/>
+    <mergeCell ref="V1:X1"/>
+    <mergeCell ref="AH1:AJ1"/>
     <mergeCell ref="J31:K31"/>
     <mergeCell ref="AN31:AO31"/>
     <mergeCell ref="AT1:AV1"/>
@@ -26508,11 +26405,14 @@
     <mergeCell ref="AN28:AO28"/>
     <mergeCell ref="J30:K30"/>
     <mergeCell ref="AN30:AO30"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="H1:K1"/>
-    <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="V1:X1"/>
-    <mergeCell ref="AH1:AJ1"/>
+    <mergeCell ref="AN36:AO36"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="AN32:AO32"/>
+    <mergeCell ref="AN33:AO33"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="AN34:AO34"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="AN35:AO35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -26521,7 +26421,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5CEA0AF-E119-44D9-BA2E-23825B943F22}">
   <dimension ref="B2:N125"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="2" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="2.140625" bestFit="1" customWidth="1"/>
@@ -26530,7 +26430,7 @@
     <col min="14" max="14" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:14" ht="15.75">
       <c r="B2" s="36" t="s">
         <v>12</v>
       </c>
@@ -26550,7 +26450,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:14" ht="15.75">
       <c r="B3" s="62">
         <v>8</v>
       </c>
@@ -26570,7 +26470,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="4" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:14" ht="15.75">
       <c r="B4" s="62">
         <v>8</v>
       </c>
@@ -26594,7 +26494,7 @@
       </c>
       <c r="K4" s="192"/>
     </row>
-    <row r="5" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:14" ht="15.75">
       <c r="B5" s="62">
         <v>8</v>
       </c>
@@ -26618,7 +26518,7 @@
       </c>
       <c r="K5" s="192"/>
     </row>
-    <row r="6" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:14" ht="15.75">
       <c r="B6" s="62">
         <v>8</v>
       </c>
@@ -26645,7 +26545,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="7" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" ht="15.75">
       <c r="B7" s="62">
         <v>8</v>
       </c>
@@ -26672,7 +26572,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="8" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:14" ht="15.75">
       <c r="B8" s="62">
         <v>8</v>
       </c>
@@ -26699,7 +26599,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="9" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" ht="15.75">
       <c r="B9" s="62">
         <v>8</v>
       </c>
@@ -26722,7 +26622,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="10" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:14" ht="15.75">
       <c r="B10" s="62">
         <v>8</v>
       </c>
@@ -26745,7 +26645,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="11" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:14" ht="15.75">
       <c r="B11" s="62">
         <v>8</v>
       </c>
@@ -26765,7 +26665,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="12" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:14" ht="15.75">
       <c r="B12" s="62">
         <v>8</v>
       </c>
@@ -26785,7 +26685,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="13" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" ht="15.75">
       <c r="B13" s="62">
         <v>8</v>
       </c>
@@ -26808,7 +26708,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" ht="15.75">
       <c r="B14" s="62">
         <v>8</v>
       </c>
@@ -26831,7 +26731,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:14" ht="15.75">
       <c r="B15" s="62">
         <v>8</v>
       </c>
@@ -26854,7 +26754,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="16" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:14" ht="15.75">
       <c r="B16" s="62">
         <v>8</v>
       </c>
@@ -26877,7 +26777,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="17" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:10" ht="15.75">
       <c r="B17" s="62">
         <v>8</v>
       </c>
@@ -26900,7 +26800,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="18" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:10" ht="15.75">
       <c r="B18" s="62">
         <v>8</v>
       </c>
@@ -26923,7 +26823,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="19" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:10" ht="15.75">
       <c r="B19" s="62">
         <v>8</v>
       </c>
@@ -26946,7 +26846,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="20" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:10" ht="15.75">
       <c r="B20" s="62">
         <v>8</v>
       </c>
@@ -26969,7 +26869,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="21" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:10" ht="15.75">
       <c r="B21" s="62">
         <v>8</v>
       </c>
@@ -26992,7 +26892,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="22" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:10" ht="15.75">
       <c r="B22" s="62">
         <v>8</v>
       </c>
@@ -27012,7 +26912,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="23" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:10" ht="15.75">
       <c r="B23" s="62">
         <v>8</v>
       </c>
@@ -27032,7 +26932,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="24" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:10" ht="15.75">
       <c r="B24" s="62">
         <v>8</v>
       </c>
@@ -27052,7 +26952,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="25" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:10" ht="15.75">
       <c r="B25" s="62">
         <v>8</v>
       </c>
@@ -27072,7 +26972,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="26" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:10" ht="15.75">
       <c r="B26" s="62">
         <v>8</v>
       </c>
@@ -27092,7 +26992,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="27" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:10" ht="15.75">
       <c r="B27" s="62">
         <v>8</v>
       </c>
@@ -27112,7 +27012,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="28" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:10" ht="15.75">
       <c r="B28" s="62">
         <v>8</v>
       </c>
@@ -27132,7 +27032,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="29" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:10" ht="15.75">
       <c r="B29" s="128">
         <v>8</v>
       </c>
@@ -27152,7 +27052,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="30" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:10" ht="15.75">
       <c r="B30" s="67">
         <v>2</v>
       </c>
@@ -27172,7 +27072,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="31" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:10" ht="15.75">
       <c r="B31" s="67">
         <v>2</v>
       </c>
@@ -27192,7 +27092,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="32" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:10" ht="15.75">
       <c r="B32" s="67">
         <v>2</v>
       </c>
@@ -27212,7 +27112,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:7" ht="15.75">
       <c r="B33" s="67">
         <v>2</v>
       </c>
@@ -27232,7 +27132,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:7" ht="15.75">
       <c r="B34" s="67">
         <v>2</v>
       </c>
@@ -27252,7 +27152,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="35" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:7" ht="15.75">
       <c r="B35" s="67">
         <v>2</v>
       </c>
@@ -27272,7 +27172,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="36" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:7" ht="15.75">
       <c r="B36" s="67">
         <v>2</v>
       </c>
@@ -27292,7 +27192,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="37" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:7" ht="15.75">
       <c r="B37" s="67">
         <v>2</v>
       </c>
@@ -27312,7 +27212,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="38" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:7" ht="15.75">
       <c r="B38" s="67">
         <v>2</v>
       </c>
@@ -27332,7 +27232,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="39" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:7" ht="15.75">
       <c r="B39" s="67">
         <v>2</v>
       </c>
@@ -27352,7 +27252,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="40" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:7" ht="15.75">
       <c r="B40" s="67">
         <v>2</v>
       </c>
@@ -27372,7 +27272,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="41" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:7" ht="15.75">
       <c r="B41" s="67">
         <v>2</v>
       </c>
@@ -27392,7 +27292,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="42" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:7" ht="15.75">
       <c r="B42" s="67">
         <v>2</v>
       </c>
@@ -27412,7 +27312,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="43" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:7" ht="15.75">
       <c r="B43" s="67">
         <v>2</v>
       </c>
@@ -27432,7 +27332,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="44" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:7" ht="15.75">
       <c r="B44" s="67">
         <v>2</v>
       </c>
@@ -27452,7 +27352,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="45" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:7" ht="15.75">
       <c r="B45" s="67">
         <v>2</v>
       </c>
@@ -27472,7 +27372,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="46" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:7" ht="15.75">
       <c r="B46" s="67">
         <v>2</v>
       </c>
@@ -27492,7 +27392,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="47" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:7" ht="15.75">
       <c r="B47" s="67">
         <v>2</v>
       </c>
@@ -27512,7 +27412,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="48" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:7" ht="15.75">
       <c r="B48" s="67">
         <v>2</v>
       </c>
@@ -27532,7 +27432,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="49" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:7" ht="15.75">
       <c r="B49" s="67">
         <v>2</v>
       </c>
@@ -27552,7 +27452,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="50" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:7" ht="15.75">
       <c r="B50" s="67">
         <v>2</v>
       </c>
@@ -27572,7 +27472,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="51" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:7" ht="15.75">
       <c r="B51" s="91">
         <v>2</v>
       </c>
@@ -27592,7 +27492,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="52" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:7" ht="15.75">
       <c r="B52" s="69">
         <v>5</v>
       </c>
@@ -27612,7 +27512,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="53" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:7" ht="15.75">
       <c r="B53" s="69">
         <v>5</v>
       </c>
@@ -27632,7 +27532,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="54" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:7" ht="15.75">
       <c r="B54" s="69">
         <v>5</v>
       </c>
@@ -27652,7 +27552,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="55" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:7" ht="15.75">
       <c r="B55" s="69">
         <v>5</v>
       </c>
@@ -27672,7 +27572,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="56" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:7" ht="15.75">
       <c r="B56" s="69">
         <v>5</v>
       </c>
@@ -27692,7 +27592,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="57" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:7" ht="15.75">
       <c r="B57" s="69">
         <v>5</v>
       </c>
@@ -27712,7 +27612,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="58" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:7" ht="15.75">
       <c r="B58" s="69">
         <v>5</v>
       </c>
@@ -27732,7 +27632,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="59" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:7" ht="15.75">
       <c r="B59" s="69">
         <v>5</v>
       </c>
@@ -27752,7 +27652,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="60" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:7" ht="15.75">
       <c r="B60" s="69">
         <v>5</v>
       </c>
@@ -27772,7 +27672,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="61" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:7" ht="15.75">
       <c r="B61" s="69">
         <v>5</v>
       </c>
@@ -27792,7 +27692,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="62" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:7" ht="15.75">
       <c r="B62" s="69">
         <v>5</v>
       </c>
@@ -27812,7 +27712,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="63" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:7" ht="15.75">
       <c r="B63" s="113">
         <v>5</v>
       </c>
@@ -27832,7 +27732,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="64" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:7" ht="15.75">
       <c r="B64" s="67">
         <v>1</v>
       </c>
@@ -27852,7 +27752,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="65" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:7" ht="15.75">
       <c r="B65" s="67">
         <v>1</v>
       </c>
@@ -27872,7 +27772,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="66" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:7" ht="15.75">
       <c r="B66" s="67">
         <v>1</v>
       </c>
@@ -27892,7 +27792,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="67" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:7" ht="15.75">
       <c r="B67" s="67">
         <v>1</v>
       </c>
@@ -27912,7 +27812,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="68" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:7" ht="15.75">
       <c r="B68" s="67">
         <v>1</v>
       </c>
@@ -27932,7 +27832,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="69" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:7" ht="15.75">
       <c r="B69" s="67">
         <v>1</v>
       </c>
@@ -27952,7 +27852,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="70" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:7" ht="15.75">
       <c r="B70" s="67">
         <v>1</v>
       </c>
@@ -27972,7 +27872,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="71" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:7" ht="15.75">
       <c r="B71" s="67">
         <v>1</v>
       </c>
@@ -27992,7 +27892,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="72" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:7" ht="15.75">
       <c r="B72" s="67">
         <v>1</v>
       </c>
@@ -28012,7 +27912,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="73" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:7" ht="15.75">
       <c r="B73" s="67">
         <v>1</v>
       </c>
@@ -28032,7 +27932,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="74" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:7" ht="15.75">
       <c r="B74" s="67">
         <v>1</v>
       </c>
@@ -28052,7 +27952,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="75" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:7" ht="15.75">
       <c r="B75" s="67">
         <v>1</v>
       </c>
@@ -28072,7 +27972,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="76" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:7" ht="15.75">
       <c r="B76" s="67">
         <v>1</v>
       </c>
@@ -28092,7 +27992,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="77" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:7" ht="15.75">
       <c r="B77" s="67">
         <v>1</v>
       </c>
@@ -28112,7 +28012,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="78" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:7" ht="15.75">
       <c r="B78" s="67">
         <v>1</v>
       </c>
@@ -28132,7 +28032,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="79" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:7" ht="15.75">
       <c r="B79" s="67">
         <v>1</v>
       </c>
@@ -28152,7 +28052,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="80" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:7" ht="15.75">
       <c r="B80" s="67">
         <v>1</v>
       </c>
@@ -28172,7 +28072,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="81" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:7" ht="15.75">
       <c r="B81" s="67">
         <v>1</v>
       </c>
@@ -28192,7 +28092,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="82" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:7" ht="15.75">
       <c r="B82" s="67">
         <v>1</v>
       </c>
@@ -28212,7 +28112,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="83" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:7" ht="15.75">
       <c r="B83" s="67">
         <v>1</v>
       </c>
@@ -28232,7 +28132,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="84" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:7" ht="15.75">
       <c r="B84" s="67">
         <v>1</v>
       </c>
@@ -28252,7 +28152,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="85" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:7" ht="15.75">
       <c r="B85" s="67">
         <v>1</v>
       </c>
@@ -28272,7 +28172,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="86" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:7" ht="15.75">
       <c r="B86" s="67">
         <v>1</v>
       </c>
@@ -28292,7 +28192,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="87" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:7" ht="15.75">
       <c r="B87" s="67">
         <v>1</v>
       </c>
@@ -28312,7 +28212,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="88" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:7" ht="15.75">
       <c r="B88" s="67">
         <v>1</v>
       </c>
@@ -28332,7 +28232,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="89" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:7" ht="15.75">
       <c r="B89" s="91">
         <v>1</v>
       </c>
@@ -28352,7 +28252,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="90" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:7" ht="15.75">
       <c r="B90" s="74">
         <v>4</v>
       </c>
@@ -28372,7 +28272,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="91" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:7" ht="15.75">
       <c r="B91" s="67">
         <v>4</v>
       </c>
@@ -28392,7 +28292,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="92" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:7" ht="15.75">
       <c r="B92" s="67">
         <v>4</v>
       </c>
@@ -28412,7 +28312,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="93" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:7" ht="15.75">
       <c r="B93" s="67">
         <v>4</v>
       </c>
@@ -28432,7 +28332,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="94" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:7" ht="15.75">
       <c r="B94" s="67">
         <v>4</v>
       </c>
@@ -28452,7 +28352,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="95" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:7" ht="15.75">
       <c r="B95" s="67">
         <v>4</v>
       </c>
@@ -28472,7 +28372,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="96" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:7" ht="15.75">
       <c r="B96" s="67">
         <v>4</v>
       </c>
@@ -28492,7 +28392,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="97" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:7" ht="15.75">
       <c r="B97" s="67">
         <v>4</v>
       </c>
@@ -28512,7 +28412,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="98" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:7" ht="15.75">
       <c r="B98" s="67">
         <v>4</v>
       </c>
@@ -28532,7 +28432,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="99" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:7" ht="15.75">
       <c r="B99" s="67">
         <v>4</v>
       </c>
@@ -28552,7 +28452,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="100" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:7" ht="15.75">
       <c r="B100" s="67">
         <v>4</v>
       </c>
@@ -28572,7 +28472,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="101" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:7" ht="15.75">
       <c r="B101" s="67">
         <v>4</v>
       </c>
@@ -28592,7 +28492,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="102" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:7" ht="15.75">
       <c r="B102" s="67">
         <v>4</v>
       </c>
@@ -28612,7 +28512,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="103" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:7" ht="15.75">
       <c r="B103" s="67">
         <v>4</v>
       </c>
@@ -28632,7 +28532,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="104" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:7" ht="15.75">
       <c r="B104" s="67">
         <v>4</v>
       </c>
@@ -28652,7 +28552,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="105" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:7" ht="15.75">
       <c r="B105" s="67">
         <v>4</v>
       </c>
@@ -28672,7 +28572,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="106" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:7" ht="15.75">
       <c r="B106" s="91">
         <v>4</v>
       </c>
@@ -28692,7 +28592,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="107" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:7" ht="15.75">
       <c r="B107" s="67">
         <v>4</v>
       </c>
@@ -28712,7 +28612,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="108" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:7" ht="15.75">
       <c r="B108" s="81">
         <v>4</v>
       </c>
@@ -28732,7 +28632,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="109" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:7" ht="15.75">
       <c r="B109" s="67">
         <v>4</v>
       </c>
@@ -28752,7 +28652,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="110" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:7" ht="15.75">
       <c r="B110" s="67">
         <v>4</v>
       </c>
@@ -28772,7 +28672,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="111" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:7" ht="15.75">
       <c r="B111" s="67">
         <v>4</v>
       </c>
@@ -28792,7 +28692,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="112" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:7" ht="15.75">
       <c r="B112" s="67">
         <v>4</v>
       </c>
@@ -28812,7 +28712,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="113" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:7" ht="15.75">
       <c r="B113" s="67">
         <v>4</v>
       </c>
@@ -28832,7 +28732,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="114" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:7" ht="15.75">
       <c r="B114" s="67">
         <v>4</v>
       </c>
@@ -28852,7 +28752,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="115" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:7" ht="15.75">
       <c r="B115" s="67">
         <v>4</v>
       </c>
@@ -28872,7 +28772,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="116" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:7" ht="15.75">
       <c r="B116" s="67">
         <v>4</v>
       </c>
@@ -28892,7 +28792,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="117" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:7" ht="15.75">
       <c r="B117" s="81">
         <v>4</v>
       </c>
@@ -28912,7 +28812,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="118" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:7" ht="15.75">
       <c r="B118" s="96">
         <v>4</v>
       </c>
@@ -28932,7 +28832,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="119" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:7" ht="15.75">
       <c r="B119" s="67">
         <v>6</v>
       </c>
@@ -28952,7 +28852,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="120" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:7" ht="15.75">
       <c r="B120" s="67">
         <v>6</v>
       </c>
@@ -28972,7 +28872,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="121" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:7" ht="15.75">
       <c r="B121" s="91">
         <v>6</v>
       </c>
@@ -28992,7 +28892,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="122" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:7" ht="15.75">
       <c r="B122" s="81">
         <v>3</v>
       </c>
@@ -29012,7 +28912,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="123" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:7" ht="15.75">
       <c r="B123" s="81">
         <v>3</v>
       </c>
@@ -29032,7 +28932,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="124" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:7" ht="15.75">
       <c r="B124" s="81">
         <v>3</v>
       </c>
@@ -29052,7 +28952,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="125" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:7" ht="15.75">
       <c r="B125" s="96">
         <v>3</v>
       </c>
@@ -29087,14 +28987,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E816FC1-7440-48FC-B2B7-E93F8C64F4FE}">
   <dimension ref="A3:I19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="1.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9">
       <c r="B3" s="142" t="s">
         <v>679</v>
       </c>
@@ -29120,7 +29020,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9">
       <c r="B4" s="142" t="s">
         <v>679</v>
       </c>
@@ -29144,7 +29044,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9">
       <c r="B5" s="142" t="s">
         <v>679</v>
       </c>
@@ -29168,7 +29068,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9">
       <c r="B6" s="142" t="s">
         <v>679</v>
       </c>
@@ -29192,7 +29092,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9">
       <c r="B7" s="142" t="s">
         <v>679</v>
       </c>
@@ -29216,7 +29116,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9">
       <c r="B8" s="142" t="s">
         <v>679</v>
       </c>
@@ -29240,7 +29140,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9">
       <c r="B9" s="142" t="s">
         <v>679</v>
       </c>
@@ -29266,7 +29166,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9">
       <c r="B10" s="142" t="s">
         <v>679</v>
       </c>
@@ -29292,27 +29192,27 @@
         <v>679</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9">
       <c r="A15" t="s">
         <v>622</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9">
       <c r="A16" t="s">
         <v>623</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1">
       <c r="A17" t="s">
         <v>624</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1">
       <c r="A18" t="s">
         <v>674</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1">
       <c r="A19" t="s">
         <v>673</v>
       </c>
@@ -29332,7 +29232,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF5BA14E-0B97-4562-826A-12019653AF3B}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -29341,7 +29241,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F842CC77-02EE-4E6C-8E0B-BD43B4A7F5EC}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>